<commit_message>
auto: 작업 자동 저장 2026-09-07 13:12
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/eval-runner/orchestrator/results/전달함_팀장님/CI_성적_Vertex_4열비교집계.xlsx
+++ b/eval-runner/orchestrator/results/전달함_팀장님/CI_성적_Vertex_4열비교집계.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4열 비교" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="유형별 분해" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -435,7 +436,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
@@ -918,7 +918,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
@@ -952,6 +951,591 @@
       <c r="B22" t="inlineStr">
         <is>
           <t>디지털 파서 무료 · 976쿼리 무료 한도 내 · 추가 청구 0 (Layout Parser 판은 ≈$70, 미실시)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>답변 합격 분해 — 비E형 447문항 · 5판 같은 문항 · 값 = 합격 문항 수 (비율) · n = 그 줄의 문항 수(비율의 분모)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>유형</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>자사 r4</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>자사 r5</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Vertex 기본값</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Vertex 옵션 변경</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>Vertex 자체 문서</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>사실확인</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>122</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>92 (75%)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>93 (76%)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>59 (48%)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>80 (66%)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>91 (75%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>절차</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>98</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>76 (78%)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>77 (79%)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>51 (52%)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>57 (58%)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>73 (74%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>조건</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>87</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>69 (79%)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>69 (79%)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>49 (56%)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>61 (70%)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>73 (84%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>가부</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>72</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>59 (82%)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>61 (85%)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>43 (60%)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>55 (76%)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>58 (81%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>수치</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>43</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>29 (67%)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>24 (56%)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>19 (44%)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>25 (58%)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>25 (58%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>정의</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>25</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>23 (92%)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>20 (80%)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>13 (52%)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>19 (76%)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>22 (88%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>정답 출처</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>자사 r4</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>자사 r5</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>Vertex 기본값</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>Vertex 옵션 변경</t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
+          <t>Vertex 자체 문서</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>매뉴얼</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>239</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>190 (79%)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>191 (80%)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>133 (56%)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>170 (71%)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>196 (82%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>출처 불명</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>140</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>103 (74%)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>97 (69%)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>68 (49%)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>83 (59%)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>89 (64%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>FAQ</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>68</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>55 (81%)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>56 (82%)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>33 (49%)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>44 (65%)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>57 (84%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>정답 근거 형태</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>자사 r4</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>자사 r5</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>Vertex 기본값</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>Vertex 옵션 변경</t>
+        </is>
+      </c>
+      <c r="G16" s="1" t="inlineStr">
+        <is>
+          <t>Vertex 자체 문서</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>문장</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>180</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>147 (82%)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>145 (81%)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>94 (52%)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>121 (67%)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>145 (81%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>출처 불명</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>140</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>103 (74%)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>97 (69%)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>68 (49%)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>83 (59%)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>89 (64%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>표 안</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>127</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>98 (77%)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>102 (80%)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>72 (57%)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>93 (73%)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>108 (85%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>읽는 법</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>n이 작은 줄(정의 25·수치 43)은 한 문항 차이가 2~4%p로 보이므로 n을 함께 볼 것. "출처 불명"은 정답 근거 청크가 export(v1+v2)에서 확인되지 않은 문항(쌍둥이 등) — 출처·형태 분류 불가, 합격률은 유효.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>정답 근거 형태</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>"표 안" = 정답 근거 청크가 표 형식(파이프 6개 이상) · "문장" = 표 아닌 본문. 그래프 문항은 시험지에 없음.</t>
         </is>
       </c>
     </row>

</xml_diff>